<commit_message>
feat: fitur ruang pakar
</commit_message>
<xml_diff>
--- a/datasets/case_base.xlsx
+++ b/datasets/case_base.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4102,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4508,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4740,7 +4740,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5320,7 +5320,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5378,7 +5378,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5436,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5552,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5668,7 +5668,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5842,7 +5842,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5900,7 +5900,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6074,7 +6074,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6132,7 +6132,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6306,7 +6306,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6422,7 +6422,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6538,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6712,7 +6712,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6770,7 +6770,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6886,7 +6886,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -6944,7 +6944,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7060,7 +7060,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7176,7 +7176,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7234,7 +7234,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7350,7 +7350,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7408,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7466,7 +7466,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7524,7 +7524,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7582,7 +7582,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -7988,7 +7988,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8046,7 +8046,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8104,7 +8104,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8220,7 +8220,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8452,7 +8452,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8510,7 +8510,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8568,7 +8568,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8684,7 +8684,7 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8858,7 +8858,7 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9032,7 +9032,7 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9090,7 +9090,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9148,7 +9148,7 @@
       </c>
       <c r="P150" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9206,7 +9206,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9264,7 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9322,7 +9322,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9380,7 +9380,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9438,7 +9438,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9496,7 +9496,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9612,7 +9612,7 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9728,7 +9728,7 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9786,7 +9786,7 @@
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9844,7 +9844,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9902,7 +9902,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -9960,7 +9960,7 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10018,7 +10018,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10076,7 +10076,7 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10134,7 +10134,7 @@
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10250,7 +10250,7 @@
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10308,7 +10308,7 @@
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10366,7 +10366,7 @@
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10424,7 +10424,7 @@
       </c>
       <c r="P172" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10482,7 +10482,7 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10540,7 +10540,7 @@
       </c>
       <c r="P174" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10598,7 +10598,7 @@
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10656,7 +10656,7 @@
       </c>
       <c r="P176" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10714,7 +10714,7 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10772,7 +10772,7 @@
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10830,7 +10830,7 @@
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10888,7 +10888,7 @@
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -10946,7 +10946,7 @@
       </c>
       <c r="P181" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11004,7 +11004,7 @@
       </c>
       <c r="P182" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11062,7 +11062,7 @@
       </c>
       <c r="P183" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11120,7 +11120,7 @@
       </c>
       <c r="P184" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11178,7 +11178,7 @@
       </c>
       <c r="P185" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11236,7 +11236,7 @@
       </c>
       <c r="P186" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11294,7 +11294,7 @@
       </c>
       <c r="P187" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="P188" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11410,7 +11410,7 @@
       </c>
       <c r="P189" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11468,7 +11468,7 @@
       </c>
       <c r="P190" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11526,7 +11526,7 @@
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11584,7 +11584,7 @@
       </c>
       <c r="P192" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11642,7 +11642,7 @@
       </c>
       <c r="P193" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11700,7 +11700,7 @@
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11758,7 +11758,7 @@
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11816,7 +11816,7 @@
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11932,7 +11932,7 @@
       </c>
       <c r="P198" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="P199" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12048,7 +12048,7 @@
       </c>
       <c r="P200" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="P201" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12164,7 +12164,7 @@
       </c>
       <c r="P202" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12222,7 +12222,7 @@
       </c>
       <c r="P203" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12280,7 +12280,7 @@
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12338,7 +12338,7 @@
       </c>
       <c r="P205" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12396,7 +12396,7 @@
       </c>
       <c r="P206" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12454,7 +12454,7 @@
       </c>
       <c r="P207" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12512,7 +12512,7 @@
       </c>
       <c r="P208" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12570,7 +12570,7 @@
       </c>
       <c r="P209" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12628,7 +12628,7 @@
       </c>
       <c r="P210" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12686,7 +12686,7 @@
       </c>
       <c r="P211" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12744,7 +12744,7 @@
       </c>
       <c r="P212" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12802,7 +12802,7 @@
       </c>
       <c r="P213" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12860,7 +12860,7 @@
       </c>
       <c r="P214" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12918,7 +12918,7 @@
       </c>
       <c r="P215" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -12976,7 +12976,7 @@
       </c>
       <c r="P216" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13034,7 +13034,7 @@
       </c>
       <c r="P217" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13092,7 +13092,7 @@
       </c>
       <c r="P218" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13150,7 +13150,7 @@
       </c>
       <c r="P219" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13208,7 +13208,7 @@
       </c>
       <c r="P220" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13266,7 +13266,7 @@
       </c>
       <c r="P221" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13324,7 +13324,7 @@
       </c>
       <c r="P222" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13382,7 +13382,7 @@
       </c>
       <c r="P223" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13440,7 +13440,7 @@
       </c>
       <c r="P224" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13498,7 +13498,7 @@
       </c>
       <c r="P225" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13556,7 +13556,7 @@
       </c>
       <c r="P226" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13614,7 +13614,7 @@
       </c>
       <c r="P227" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13672,7 +13672,7 @@
       </c>
       <c r="P228" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13730,7 +13730,7 @@
       </c>
       <c r="P229" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="P230" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13846,7 +13846,7 @@
       </c>
       <c r="P231" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13904,7 +13904,7 @@
       </c>
       <c r="P232" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -13962,7 +13962,7 @@
       </c>
       <c r="P233" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14020,7 +14020,7 @@
       </c>
       <c r="P234" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14078,7 +14078,7 @@
       </c>
       <c r="P235" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14136,7 +14136,7 @@
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14194,7 +14194,7 @@
       </c>
       <c r="P237" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14252,7 +14252,7 @@
       </c>
       <c r="P238" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14310,7 +14310,7 @@
       </c>
       <c r="P239" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14368,7 +14368,7 @@
       </c>
       <c r="P240" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14426,7 +14426,7 @@
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14484,7 +14484,7 @@
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14542,7 +14542,7 @@
       </c>
       <c r="P243" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14600,7 +14600,7 @@
       </c>
       <c r="P244" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14658,7 +14658,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14716,7 +14716,7 @@
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14774,7 +14774,7 @@
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14832,7 +14832,7 @@
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14890,7 +14890,7 @@
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -14948,7 +14948,7 @@
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15006,7 +15006,7 @@
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15064,7 +15064,7 @@
       </c>
       <c r="P252" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15122,7 +15122,7 @@
       </c>
       <c r="P253" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15180,7 +15180,7 @@
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15238,7 +15238,7 @@
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15296,7 +15296,7 @@
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15354,7 +15354,7 @@
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15412,7 +15412,7 @@
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15470,7 +15470,7 @@
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15528,7 +15528,7 @@
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15586,7 +15586,7 @@
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15644,7 +15644,7 @@
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15702,7 +15702,7 @@
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15760,7 +15760,7 @@
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15818,7 +15818,7 @@
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15876,7 +15876,7 @@
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15934,7 +15934,7 @@
       </c>
       <c r="P267" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -15992,7 +15992,7 @@
       </c>
       <c r="P268" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16050,7 +16050,7 @@
       </c>
       <c r="P269" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16108,7 +16108,7 @@
       </c>
       <c r="P270" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16166,7 +16166,7 @@
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16282,7 +16282,7 @@
       </c>
       <c r="P273" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16340,7 +16340,7 @@
       </c>
       <c r="P274" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16398,7 +16398,7 @@
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16456,7 +16456,7 @@
       </c>
       <c r="P276" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16514,7 +16514,7 @@
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16572,7 +16572,7 @@
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16630,7 +16630,7 @@
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16688,7 +16688,7 @@
       </c>
       <c r="P280" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16746,7 +16746,7 @@
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16804,7 +16804,7 @@
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16862,7 +16862,7 @@
       </c>
       <c r="P283" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16920,7 +16920,7 @@
       </c>
       <c r="P284" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="P285" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17036,7 +17036,7 @@
       </c>
       <c r="P286" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17094,7 +17094,7 @@
       </c>
       <c r="P287" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17152,7 +17152,7 @@
       </c>
       <c r="P288" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17210,7 +17210,7 @@
       </c>
       <c r="P289" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17268,7 +17268,7 @@
       </c>
       <c r="P290" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17326,7 +17326,7 @@
       </c>
       <c r="P291" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17384,7 +17384,7 @@
       </c>
       <c r="P292" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17442,7 +17442,7 @@
       </c>
       <c r="P293" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17500,7 +17500,7 @@
       </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17558,7 +17558,7 @@
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17616,7 +17616,7 @@
       </c>
       <c r="P296" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17674,7 +17674,7 @@
       </c>
       <c r="P297" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17732,7 +17732,7 @@
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17790,7 +17790,7 @@
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17848,7 +17848,7 @@
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17906,7 +17906,7 @@
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -17964,7 +17964,7 @@
       </c>
       <c r="P302" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18022,7 +18022,7 @@
       </c>
       <c r="P303" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18080,7 +18080,7 @@
       </c>
       <c r="P304" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18138,7 +18138,7 @@
       </c>
       <c r="P305" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18196,7 +18196,7 @@
       </c>
       <c r="P306" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18254,7 +18254,7 @@
       </c>
       <c r="P307" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18312,7 +18312,7 @@
       </c>
       <c r="P308" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18370,7 +18370,7 @@
       </c>
       <c r="P309" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18428,7 +18428,7 @@
       </c>
       <c r="P310" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18486,7 +18486,7 @@
       </c>
       <c r="P311" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18544,7 +18544,7 @@
       </c>
       <c r="P312" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18602,7 +18602,7 @@
       </c>
       <c r="P313" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18660,7 +18660,7 @@
       </c>
       <c r="P314" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18718,7 +18718,7 @@
       </c>
       <c r="P315" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18776,7 +18776,7 @@
       </c>
       <c r="P316" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18834,7 +18834,7 @@
       </c>
       <c r="P317" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18892,7 +18892,7 @@
       </c>
       <c r="P318" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -18950,7 +18950,7 @@
       </c>
       <c r="P319" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19008,7 +19008,7 @@
       </c>
       <c r="P320" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19066,7 +19066,7 @@
       </c>
       <c r="P321" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19124,7 +19124,7 @@
       </c>
       <c r="P322" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19182,7 +19182,7 @@
       </c>
       <c r="P323" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19240,7 +19240,7 @@
       </c>
       <c r="P324" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19298,7 +19298,7 @@
       </c>
       <c r="P325" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19356,7 +19356,7 @@
       </c>
       <c r="P326" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19414,7 +19414,7 @@
       </c>
       <c r="P327" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19472,7 @@
       </c>
       <c r="P328" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19530,7 +19530,7 @@
       </c>
       <c r="P329" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19588,7 +19588,7 @@
       </c>
       <c r="P330" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19646,7 +19646,7 @@
       </c>
       <c r="P331" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19704,7 +19704,7 @@
       </c>
       <c r="P332" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19762,7 +19762,7 @@
       </c>
       <c r="P333" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19820,7 +19820,7 @@
       </c>
       <c r="P334" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19878,7 +19878,7 @@
       </c>
       <c r="P335" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19936,7 +19936,7 @@
       </c>
       <c r="P336" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -19994,7 +19994,7 @@
       </c>
       <c r="P337" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20052,7 +20052,7 @@
       </c>
       <c r="P338" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20110,7 +20110,7 @@
       </c>
       <c r="P339" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20168,7 +20168,7 @@
       </c>
       <c r="P340" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20226,7 +20226,7 @@
       </c>
       <c r="P341" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20284,7 +20284,7 @@
       </c>
       <c r="P342" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20342,7 @@
       </c>
       <c r="P343" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20400,7 +20400,7 @@
       </c>
       <c r="P344" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20458,7 +20458,7 @@
       </c>
       <c r="P345" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20516,7 +20516,7 @@
       </c>
       <c r="P346" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20574,7 +20574,7 @@
       </c>
       <c r="P347" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20632,7 +20632,7 @@
       </c>
       <c r="P348" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20690,7 +20690,7 @@
       </c>
       <c r="P349" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20748,7 +20748,7 @@
       </c>
       <c r="P350" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20806,7 +20806,7 @@
       </c>
       <c r="P351" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20864,7 +20864,7 @@
       </c>
       <c r="P352" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20922,7 +20922,7 @@
       </c>
       <c r="P353" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -20980,7 +20980,7 @@
       </c>
       <c r="P354" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21038,7 +21038,7 @@
       </c>
       <c r="P355" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21096,7 +21096,7 @@
       </c>
       <c r="P356" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21154,7 +21154,7 @@
       </c>
       <c r="P357" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21212,7 +21212,7 @@
       </c>
       <c r="P358" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21270,7 +21270,7 @@
       </c>
       <c r="P359" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21328,7 +21328,7 @@
       </c>
       <c r="P360" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21386,7 +21386,7 @@
       </c>
       <c r="P361" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21444,7 +21444,7 @@
       </c>
       <c r="P362" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21502,7 +21502,7 @@
       </c>
       <c r="P363" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21560,7 +21560,7 @@
       </c>
       <c r="P364" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21618,7 +21618,7 @@
       </c>
       <c r="P365" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21676,7 +21676,7 @@
       </c>
       <c r="P366" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21734,7 +21734,7 @@
       </c>
       <c r="P367" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21792,7 +21792,7 @@
       </c>
       <c r="P368" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21850,7 +21850,7 @@
       </c>
       <c r="P369" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21908,7 +21908,7 @@
       </c>
       <c r="P370" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -21966,7 +21966,7 @@
       </c>
       <c r="P371" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22024,7 +22024,7 @@
       </c>
       <c r="P372" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22082,7 +22082,7 @@
       </c>
       <c r="P373" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22140,7 +22140,7 @@
       </c>
       <c r="P374" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22198,7 +22198,7 @@
       </c>
       <c r="P375" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22256,7 +22256,7 @@
       </c>
       <c r="P376" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22314,7 +22314,7 @@
       </c>
       <c r="P377" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22372,7 +22372,7 @@
       </c>
       <c r="P378" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22430,7 +22430,7 @@
       </c>
       <c r="P379" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22488,7 +22488,7 @@
       </c>
       <c r="P380" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22546,7 +22546,7 @@
       </c>
       <c r="P381" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22604,7 +22604,7 @@
       </c>
       <c r="P382" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22662,7 +22662,7 @@
       </c>
       <c r="P383" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22720,7 +22720,7 @@
       </c>
       <c r="P384" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22778,7 +22778,7 @@
       </c>
       <c r="P385" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22836,7 +22836,7 @@
       </c>
       <c r="P386" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22894,7 +22894,7 @@
       </c>
       <c r="P387" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -22952,7 +22952,7 @@
       </c>
       <c r="P388" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23010,7 +23010,7 @@
       </c>
       <c r="P389" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23068,7 +23068,7 @@
       </c>
       <c r="P390" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23126,7 +23126,7 @@
       </c>
       <c r="P391" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23184,7 +23184,7 @@
       </c>
       <c r="P392" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23242,7 +23242,7 @@
       </c>
       <c r="P393" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23300,7 +23300,7 @@
       </c>
       <c r="P394" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23358,7 +23358,7 @@
       </c>
       <c r="P395" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>
@@ -23416,7 +23416,7 @@
       </c>
       <c r="P396" t="inlineStr">
         <is>
-          <t>2026-06-16 12:19:53</t>
+          <t>2026-06-16 16:32:39</t>
         </is>
       </c>
     </row>

</xml_diff>